<commit_message>
Actualizar datos desde planilla Excel 1C 2026
</commit_message>
<xml_diff>
--- a/Presencialidad 1C 2026.xlsx
+++ b/Presencialidad 1C 2026.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="9000" tabRatio="500"/>
+    <workbookView windowWidth="27947" windowHeight="12240" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -174,6 +174,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
       <t>Administraci</t>
     </r>
     <r>
@@ -289,6 +295,9 @@
     <t>Seminario de Actualización en Tecnologías Web</t>
   </si>
   <si>
+    <t>Eckerdt</t>
+  </si>
+  <si>
     <t>Liderazgo y Gestión de Equipos</t>
   </si>
   <si>
@@ -344,6 +353,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Modelizado de </t>
     </r>
     <r>
@@ -400,9 +415,6 @@
   </si>
   <si>
     <t>Romitelli</t>
-  </si>
-  <si>
-    <t>Iberti</t>
   </si>
   <si>
     <t>PP2 Desarrollo de Sistemas de Información Orientados a la Gestión y Apoyo a las Decisiones</t>
@@ -1072,7 +1084,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1081,9 +1093,6 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1886,22 +1895,22 @@
         <v>38</v>
       </c>
       <c r="D20" s="4"/>
-      <c r="E20" s="5" t="s">
+      <c r="E20" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5" t="s">
+      <c r="F20" s="1"/>
+      <c r="G20" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5" t="s">
+      <c r="H20" s="1"/>
+      <c r="I20" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="J20" s="5"/>
-      <c r="K20" s="5" t="s">
+      <c r="J20" s="1"/>
+      <c r="K20" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="L20" s="5"/>
+      <c r="L20" s="1"/>
     </row>
     <row r="21" spans="1:17">
       <c r="C21" s="2" t="s">
@@ -1948,22 +1957,22 @@
       <c r="E22" t="s">
         <v>47</v>
       </c>
-      <c r="F22" s="6" t="s">
+      <c r="F22" s="5" t="s">
         <v>48</v>
       </c>
       <c r="G22" t="s">
         <v>47</v>
       </c>
-      <c r="H22" s="6" t="s">
+      <c r="H22" s="5" t="s">
         <v>48</v>
       </c>
       <c r="I22" t="s">
         <v>49</v>
       </c>
-      <c r="J22" s="6" t="s">
+      <c r="J22" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="K22" s="6" t="s">
+      <c r="K22" s="5" t="s">
         <v>51</v>
       </c>
       <c r="L22" t="s">
@@ -2003,7 +2012,7 @@
       <c r="I24" t="s">
         <v>59</v>
       </c>
-      <c r="J24" s="7" t="s">
+      <c r="J24" s="6" t="s">
         <v>60</v>
       </c>
       <c r="K24" t="s">
@@ -2052,7 +2061,7 @@
       <c r="B26" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="6" t="s">
         <v>73</v>
       </c>
       <c r="D26" t="s">
@@ -2070,7 +2079,7 @@
       <c r="H26" t="s">
         <v>78</v>
       </c>
-      <c r="I26" s="7" t="s">
+      <c r="I26" s="6" t="s">
         <v>79</v>
       </c>
       <c r="J26" t="s">
@@ -2084,7 +2093,7 @@
       </c>
     </row>
     <row r="27" spans="1:17">
-      <c r="E27" s="7" t="s">
+      <c r="E27" s="6" t="s">
         <v>73</v>
       </c>
       <c r="F27" t="s">
@@ -2102,42 +2111,42 @@
         <v>7</v>
       </c>
       <c r="C28" t="s">
-        <v>47</v>
+        <v>83</v>
       </c>
       <c r="D28" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E28" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F28" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G28" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H28" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="I28" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J28" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K28" t="s">
         <v>47</v>
       </c>
       <c r="L28" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="29" spans="1:17">
       <c r="G29" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H29" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="30" spans="1:17">
@@ -2145,7 +2154,7 @@
         <v>8</v>
       </c>
       <c r="C30" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D30" t="s">
         <v>52</v>
@@ -2154,22 +2163,22 @@
         <v>67</v>
       </c>
       <c r="F30" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G30" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H30" t="s">
         <v>46</v>
       </c>
       <c r="I30" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J30" t="s">
         <v>50</v>
       </c>
       <c r="K30" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="L30" t="s">
         <v>46</v>
@@ -2180,15 +2189,15 @@
         <v>67</v>
       </c>
       <c r="H31" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="32" spans="1:17">
       <c r="B32" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C32" s="7" t="s">
-        <v>94</v>
+      <c r="C32" s="6" t="s">
+        <v>95</v>
       </c>
       <c r="D32" t="s">
         <v>54</v>
@@ -2197,16 +2206,16 @@
         <v>63</v>
       </c>
       <c r="F32" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G32" t="s">
         <v>59</v>
       </c>
       <c r="H32" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I32" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="J32" t="s">
         <v>72</v>
@@ -2215,7 +2224,7 @@
         <v>63</v>
       </c>
       <c r="L32" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="33" spans="2:12">
@@ -2223,42 +2232,42 @@
         <v>10</v>
       </c>
       <c r="C33" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D33" t="s">
         <v>76</v>
       </c>
-      <c r="E33" s="6" t="s">
-        <v>99</v>
+      <c r="E33" s="5" t="s">
+        <v>100</v>
       </c>
       <c r="F33" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G33" t="s">
         <v>63</v>
       </c>
-      <c r="H33" s="6" t="s">
+      <c r="H33" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="I33" t="s">
+        <v>103</v>
+      </c>
+      <c r="J33" t="s">
+        <v>104</v>
+      </c>
+      <c r="K33" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="L33" t="s">
         <v>101</v>
-      </c>
-      <c r="I33" t="s">
-        <v>102</v>
-      </c>
-      <c r="J33" t="s">
-        <v>103</v>
-      </c>
-      <c r="K33" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="L33" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="34" spans="2:12">
       <c r="E34" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F34" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="35" spans="2:12">
@@ -2266,31 +2275,31 @@
         <v>11</v>
       </c>
       <c r="C35" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D35" t="s">
+        <v>106</v>
+      </c>
+      <c r="E35" t="s">
         <v>105</v>
       </c>
-      <c r="E35" t="s">
-        <v>104</v>
-      </c>
       <c r="F35" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G35" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H35" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I35" t="s">
         <v>61</v>
       </c>
       <c r="J35" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K35" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L35" t="s">
         <v>80</v>
@@ -2301,7 +2310,7 @@
         <v>61</v>
       </c>
       <c r="L36" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="37" spans="2:12">
@@ -2309,34 +2318,34 @@
         <v>12</v>
       </c>
       <c r="C37" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D37" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E37" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F37" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G37" t="s">
         <v>45</v>
       </c>
       <c r="H37" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="I37" t="s">
         <v>45</v>
       </c>
       <c r="J37" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="K37" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L37" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="38" spans="2:12">
@@ -2350,7 +2359,7 @@
         <v>46</v>
       </c>
       <c r="E38" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F38" t="s">
         <v>52</v>
@@ -2362,10 +2371,10 @@
         <v>46</v>
       </c>
       <c r="I38" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J38" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="K38" t="s">
         <v>59</v>
@@ -2376,10 +2385,10 @@
     </row>
     <row r="39" spans="2:12">
       <c r="G39" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H39" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="40" spans="2:12">
@@ -2387,31 +2396,31 @@
         <v>14</v>
       </c>
       <c r="C40" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D40" t="s">
         <v>56</v>
       </c>
       <c r="E40" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F40" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G40" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H40" t="s">
         <v>54</v>
       </c>
       <c r="I40" t="s">
-        <v>117</v>
+        <v>57</v>
       </c>
       <c r="J40" t="s">
         <v>58</v>
       </c>
       <c r="K40" t="s">
-        <v>117</v>
+        <v>57</v>
       </c>
       <c r="L40" t="s">
         <v>62</v>
@@ -2419,7 +2428,7 @@
     </row>
     <row r="41" spans="2:12">
       <c r="K41" t="s">
-        <v>117</v>
+        <v>57</v>
       </c>
       <c r="L41" t="s">
         <v>58</v>
@@ -2432,7 +2441,7 @@
       <c r="C42" t="s">
         <v>77</v>
       </c>
-      <c r="D42" s="8" t="s">
+      <c r="D42" s="7" t="s">
         <v>118</v>
       </c>
       <c r="E42" t="s">
@@ -2531,10 +2540,10 @@
         <v>128</v>
       </c>
       <c r="D46" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E46" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F46" t="s">
         <v>129</v>
@@ -2542,11 +2551,11 @@
       <c r="G46" t="s">
         <v>130</v>
       </c>
-      <c r="H46" s="6" t="s">
+      <c r="H46" s="5" t="s">
         <v>80</v>
       </c>
       <c r="I46" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J46" t="s">
         <v>76</v>
@@ -2554,10 +2563,10 @@
     </row>
     <row r="47" spans="2:12">
       <c r="G47" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H47" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update schedule data from latest spreadsheet
</commit_message>
<xml_diff>
--- a/Presencialidad 1C 2026.xlsx
+++ b/Presencialidad 1C 2026.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="131">
   <si>
     <t>Presencialidad 1C 2026</t>
   </si>
@@ -405,7 +405,7 @@
     <t>Odstrcil</t>
   </si>
   <si>
-    <t>Cefail</t>
+    <t>Cefali</t>
   </si>
   <si>
     <t>Murua</t>
@@ -1553,6 +1553,9 @@
       <c r="G6" t="s">
         <v>20</v>
       </c>
+      <c r="L6" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="7" spans="1:17">
       <c r="A7" s="3">
@@ -1748,6 +1751,9 @@
       </c>
       <c r="G14" t="s">
         <v>20</v>
+      </c>
+      <c r="L14" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:17">

</xml_diff>

<commit_message>
Update schedule data based on user modifications
</commit_message>
<xml_diff>
--- a/Presencialidad 1C 2026.xlsx
+++ b/Presencialidad 1C 2026.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="9000" tabRatio="500"/>
+    <workbookView windowWidth="27947" windowHeight="12240" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1516,6 +1516,9 @@
       <c r="B4" t="s">
         <v>22</v>
       </c>
+      <c r="L4" t="s">
+        <v>21</v>
+      </c>
       <c r="M4" t="s">
         <v>19</v>
       </c>
@@ -1553,9 +1556,6 @@
       <c r="G6" t="s">
         <v>20</v>
       </c>
-      <c r="L6" t="s">
-        <v>21</v>
-      </c>
     </row>
     <row r="7" spans="1:17">
       <c r="A7" s="3">
@@ -1715,6 +1715,9 @@
       <c r="B12" t="s">
         <v>31</v>
       </c>
+      <c r="L12" t="s">
+        <v>21</v>
+      </c>
       <c r="M12" t="s">
         <v>19</v>
       </c>
@@ -1751,9 +1754,6 @@
       </c>
       <c r="G14" t="s">
         <v>20</v>
-      </c>
-      <c r="L14" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:17">

</xml_diff>

<commit_message>
Actualizar datos de presencialidad y archivos relacionados
</commit_message>
<xml_diff>
--- a/Presencialidad 1C 2026.xlsx
+++ b/Presencialidad 1C 2026.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27947" windowHeight="12240" tabRatio="500"/>
+    <workbookView windowWidth="27947" windowHeight="11640" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -331,7 +331,7 @@
     <t>Capara</t>
   </si>
   <si>
-    <t>Blumenkranz</t>
+    <t>Cendra</t>
   </si>
   <si>
     <t>Desarrollo de Sistemas de Inteligencia Artificial</t>

</xml_diff>

<commit_message>
Update data from Excel
</commit_message>
<xml_diff>
--- a/Presencialidad 1C 2026.xlsx
+++ b/Presencialidad 1C 2026.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27947" windowHeight="11640" tabRatio="500"/>
+    <workbookView windowWidth="22188" windowHeight="8400" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2263,8 +2263,8 @@
       </c>
     </row>
     <row r="34" spans="2:12">
-      <c r="E34" t="s">
-        <v>103</v>
+      <c r="E34" s="5" t="s">
+        <v>100</v>
       </c>
       <c r="F34" t="s">
         <v>104</v>

</xml_diff>

<commit_message>
Update data from Excel - second iteration
</commit_message>
<xml_diff>
--- a/Presencialidad 1C 2026.xlsx
+++ b/Presencialidad 1C 2026.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="8400" tabRatio="500"/>
+    <workbookView windowWidth="27947" windowHeight="12240" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -378,6 +378,9 @@
     <t>Procesamiento de Aprendizaje Automático</t>
   </si>
   <si>
+    <t>Seminario de Actualización</t>
+  </si>
+  <si>
     <t>Pita</t>
   </si>
   <si>
@@ -394,9 +397,6 @@
   </si>
   <si>
     <t>Técnicas de Procesamiento Digital de Imágenes</t>
-  </si>
-  <si>
-    <t>Seminario de Actualización</t>
   </si>
   <si>
     <t>Gonzalez</t>
@@ -2267,7 +2267,7 @@
         <v>100</v>
       </c>
       <c r="F34" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="35" spans="2:12">
@@ -2275,31 +2275,31 @@
         <v>11</v>
       </c>
       <c r="C35" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D35" t="s">
+        <v>107</v>
+      </c>
+      <c r="E35" t="s">
         <v>106</v>
       </c>
-      <c r="E35" t="s">
-        <v>105</v>
-      </c>
       <c r="F35" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="G35" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H35" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I35" t="s">
         <v>61</v>
       </c>
       <c r="J35" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="L35" t="s">
         <v>80</v>
@@ -2310,7 +2310,7 @@
         <v>61</v>
       </c>
       <c r="L36" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="37" spans="2:12">
@@ -2333,19 +2333,19 @@
         <v>45</v>
       </c>
       <c r="H37" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I37" t="s">
         <v>45</v>
       </c>
       <c r="J37" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K37" t="s">
         <v>100</v>
       </c>
       <c r="L37" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
     </row>
     <row r="38" spans="2:12">
@@ -2566,7 +2566,7 @@
         <v>103</v>
       </c>
       <c r="H47" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data from Excel - third iteration
</commit_message>
<xml_diff>
--- a/Presencialidad 1C 2026.xlsx
+++ b/Presencialidad 1C 2026.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="131">
   <si>
     <t>Presencialidad 1C 2026</t>
   </si>
@@ -2323,12 +2323,8 @@
       <c r="D37" t="s">
         <v>86</v>
       </c>
-      <c r="E37" t="s">
-        <v>100</v>
-      </c>
-      <c r="F37" t="s">
-        <v>86</v>
-      </c>
+      <c r="E37"/>
+      <c r="F37"/>
       <c r="G37" t="s">
         <v>45</v>
       </c>
@@ -2340,12 +2336,6 @@
       </c>
       <c r="J37" t="s">
         <v>111</v>
-      </c>
-      <c r="K37" t="s">
-        <v>100</v>
-      </c>
-      <c r="L37" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="38" spans="2:12">

</xml_diff>

<commit_message>
Update data from Excel - fourth iteration
</commit_message>
<xml_diff>
--- a/Presencialidad 1C 2026.xlsx
+++ b/Presencialidad 1C 2026.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="133">
   <si>
     <t>Presencialidad 1C 2026</t>
   </si>
@@ -217,7 +217,7 @@
     <t>Inglés</t>
   </si>
   <si>
-    <t>A definir</t>
+    <t>Villariño</t>
   </si>
   <si>
     <t>Desarrollo de Sistemas Orientado a Objetos</t>
@@ -415,6 +415,12 @@
   </si>
   <si>
     <t>Romitelli</t>
+  </si>
+  <si>
+    <t>Mercado</t>
+  </si>
+  <si>
+    <t>Malvacio</t>
   </si>
   <si>
     <t>PP2 Desarrollo de Sistemas de Información Orientados a la Gestión y Apoyo a las Decisiones</t>
@@ -2404,13 +2410,13 @@
         <v>54</v>
       </c>
       <c r="I40" t="s">
-        <v>57</v>
+        <v>118</v>
       </c>
       <c r="J40" t="s">
         <v>58</v>
       </c>
       <c r="K40" t="s">
-        <v>57</v>
+        <v>119</v>
       </c>
       <c r="L40" t="s">
         <v>62</v>
@@ -2418,7 +2424,7 @@
     </row>
     <row r="41" spans="2:12">
       <c r="K41" t="s">
-        <v>57</v>
+        <v>118</v>
       </c>
       <c r="L41" t="s">
         <v>58</v>
@@ -2432,31 +2438,31 @@
         <v>77</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E42" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F42" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="G42" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="H42" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="I42" t="s">
         <v>77</v>
       </c>
       <c r="J42" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="K42" t="s">
         <v>65</v>
       </c>
       <c r="L42" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="43" spans="2:12">
@@ -2464,10 +2470,10 @@
         <v>65</v>
       </c>
       <c r="H43" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I43" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="J43" t="s">
         <v>72</v>
@@ -2487,25 +2493,25 @@
         <v>45</v>
       </c>
       <c r="F44" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="G44" t="s">
-        <v>57</v>
+        <v>119</v>
       </c>
       <c r="H44" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I44" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="J44" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="K44" t="s">
         <v>45</v>
       </c>
       <c r="L44" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="45" spans="2:12">
@@ -2516,10 +2522,10 @@
         <v>70</v>
       </c>
       <c r="G45" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H45" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="46" spans="2:12">
@@ -2527,7 +2533,7 @@
         <v>17</v>
       </c>
       <c r="C46" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D46" t="s">
         <v>86</v>
@@ -2536,10 +2542,10 @@
         <v>89</v>
       </c>
       <c r="F46" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="G46" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H46" s="5" t="s">
         <v>80</v>

</xml_diff>

<commit_message>
Actualización de datos desde Excel
</commit_message>
<xml_diff>
--- a/Presencialidad 1C 2026.xlsx
+++ b/Presencialidad 1C 2026.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27947" windowHeight="12240" tabRatio="500"/>
+    <workbookView windowWidth="22188" windowHeight="9000" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -399,7 +399,7 @@
     <t>Técnicas de Procesamiento Digital de Imágenes</t>
   </si>
   <si>
-    <t>Gonzalez</t>
+    <t>Salico</t>
   </si>
   <si>
     <t>Odstrcil</t>
@@ -2329,8 +2329,6 @@
       <c r="D37" t="s">
         <v>86</v>
       </c>
-      <c r="E37"/>
-      <c r="F37"/>
       <c r="G37" t="s">
         <v>45</v>
       </c>

</xml_diff>